<commit_message>
Restringe a planilha de quatro colunas aos municipios do recorte VPE
Sai Santa Cruz Cabralia, unico municipio fora do VPE com local atendido em
100 m: 487 linhas, 348 escolas, 62 municipios.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011XXDPBuJByk22LRB6WjuQf
</commit_message>
<xml_diff>
--- a/escolas_e_cameras.xlsx
+++ b/escolas_e_cameras.xlsx
@@ -446,7 +446,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:D491"/>
+  <dimension ref="A1:D488"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -8994,132 +8994,132 @@
     <row r="389">
       <c r="A389" s="2" t="inlineStr">
         <is>
-          <t>SANTA CRUZ CABRÁLIA</t>
+          <t>SANTA MARIA DA VITÓRIA</t>
         </is>
       </c>
       <c r="B389" s="2" t="inlineStr">
         <is>
-          <t>COLÉGIO ESTADUAL INDÍGENA COROA VERMELHA</t>
+          <t>UFOB - UNIVERSIDADE FEDERAL DO OESTE DA BAHIA</t>
         </is>
       </c>
       <c r="C389" s="2" t="inlineStr">
         <is>
-          <t>BR 367 KM 06 - POVOADO COROA VERMELHA</t>
+          <t>PRAÇA ARGEMIRO FILARDI, S/N - CENTRO</t>
         </is>
       </c>
       <c r="D389" s="2" t="inlineStr">
         <is>
-          <t>8B-108_LPR_COROA VERMELHA PROX AO MEMORIAL EPOP DO DESCOBRIMENTO</t>
+          <t>30-013_RF_TP_IV_TRAVESSA BRASIL SANTA MARIA DA VITORIA</t>
         </is>
       </c>
     </row>
     <row r="390">
       <c r="A390" s="2" t="inlineStr">
         <is>
-          <t>SANTA CRUZ CABRÁLIA</t>
+          <t>SANTANA</t>
         </is>
       </c>
       <c r="B390" s="2" t="inlineStr">
         <is>
-          <t>COLÉGIO ESTADUAL INDÍGENA COROA VERMELHA</t>
+          <t>PREDIO ESCOLAR BARAO DO RIO BRANCO</t>
         </is>
       </c>
       <c r="C390" s="2" t="inlineStr">
         <is>
-          <t>BR 367 KM 06 - POVOADO COROA VERMELHA</t>
+          <t>AVENIDA MANOEL NOVAIS, S/N - CENTRO</t>
         </is>
       </c>
       <c r="D390" s="2" t="inlineStr">
         <is>
-          <t>8B-109_LPR_COROA VERMELHA PROX AO MEMORIAL EPOP DO DESCOBRIMENTO</t>
+          <t>30-050_RF_TP_IV_RUA JOSE BONIFACIO</t>
         </is>
       </c>
     </row>
     <row r="391">
       <c r="A391" s="2" t="inlineStr">
         <is>
-          <t>SANTA CRUZ CABRÁLIA</t>
+          <t>SANTO AMARO</t>
         </is>
       </c>
       <c r="B391" s="2" t="inlineStr">
         <is>
-          <t>COLÉGIO ESTADUAL INDÍGENA COROA VERMELHA</t>
+          <t>APAE - SANTO AMARO</t>
         </is>
       </c>
       <c r="C391" s="2" t="inlineStr">
         <is>
-          <t>BR 367 KM 06 - POVOADO COROA VERMELHA</t>
+          <t>AV. FERREIRA BANDEIRA, S/N - CENTRO</t>
         </is>
       </c>
       <c r="D391" s="2" t="inlineStr">
         <is>
-          <t>8B-138_PTZ R TANCREDO NEVES PROXIMO AO MOTO TAXI</t>
+          <t>20-004_PTZ_AV VIANA BANDEIRA PX AO MERCADINHO LIPE FUNDO DA PREFEITURA</t>
         </is>
       </c>
     </row>
     <row r="392">
       <c r="A392" s="2" t="inlineStr">
         <is>
-          <t>SANTA MARIA DA VITÓRIA</t>
+          <t>SANTO ANTÔNIO DE JESUS</t>
         </is>
       </c>
       <c r="B392" s="2" t="inlineStr">
         <is>
-          <t>UFOB - UNIVERSIDADE FEDERAL DO OESTE DA BAHIA</t>
+          <t>CETEP - RECÔNCAVO</t>
         </is>
       </c>
       <c r="C392" s="2" t="inlineStr">
         <is>
-          <t>PRAÇA ARGEMIRO FILARDI, S/N - CENTRO</t>
+          <t>PRIMEIRA TRAVESSA DO AMPARO, S/N, ZONA URBANA</t>
         </is>
       </c>
       <c r="D392" s="2" t="inlineStr">
         <is>
-          <t>30-013_RF_TP_IV_TRAVESSA BRASIL SANTA MARIA DA VITORIA</t>
+          <t>14B-064_RF_TP_III_TV DO AMPARO - PRÓXIMO AO CETEP</t>
         </is>
       </c>
     </row>
     <row r="393">
       <c r="A393" s="2" t="inlineStr">
         <is>
-          <t>SANTANA</t>
+          <t>SANTO ANTÔNIO DE JESUS</t>
         </is>
       </c>
       <c r="B393" s="2" t="inlineStr">
         <is>
-          <t>PREDIO ESCOLAR BARAO DO RIO BRANCO</t>
+          <t>CIRETRAN</t>
         </is>
       </c>
       <c r="C393" s="2" t="inlineStr">
         <is>
-          <t>AVENIDA MANOEL NOVAIS, S/N - CENTRO</t>
+          <t>AV. ANTONIO CARLOS MAGALHAES, S/N - SÃO PAULO</t>
         </is>
       </c>
       <c r="D393" s="2" t="inlineStr">
         <is>
-          <t>30-050_RF_TP_IV_RUA JOSE BONIFACIO</t>
+          <t>14B-062_RF_TP_III_AV ANTONIO CARLOS NAGALHAES</t>
         </is>
       </c>
     </row>
     <row r="394">
       <c r="A394" s="2" t="inlineStr">
         <is>
-          <t>SANTO AMARO</t>
+          <t>SANTO ANTÔNIO DE JESUS</t>
         </is>
       </c>
       <c r="B394" s="2" t="inlineStr">
         <is>
-          <t>APAE - SANTO AMARO</t>
+          <t>PRÉDIO ESCOLAR FLORENTINO FIRMINO DE ALMEIDA</t>
         </is>
       </c>
       <c r="C394" s="2" t="inlineStr">
         <is>
-          <t>AV. FERREIRA BANDEIRA, S/N - CENTRO</t>
+          <t>AV. ANTONIO CARLOS MAGALHÃES, S/N - SÃO PAULO</t>
         </is>
       </c>
       <c r="D394" s="2" t="inlineStr">
         <is>
-          <t>20-004_PTZ_AV VIANA BANDEIRA PX AO MERCADINHO LIPE FUNDO DA PREFEITURA</t>
+          <t>14B-054_LPR_AV HEITOR LIRIO DE MELO GRANNICK MARMORES STD CENTRO</t>
         </is>
       </c>
     </row>
@@ -9131,17 +9131,17 @@
       </c>
       <c r="B395" s="2" t="inlineStr">
         <is>
-          <t>CETEP - RECÔNCAVO</t>
+          <t>UNIFACEMP - CENTRO UNIVERSITÁRIO DE CIÊNCIAS E EMPREENDEDORISMO</t>
         </is>
       </c>
       <c r="C395" s="2" t="inlineStr">
         <is>
-          <t>PRIMEIRA TRAVESSA DO AMPARO, S/N, ZONA URBANA</t>
+          <t>RUA ANTONIO VEIGA ARGOLO, N 58 - CENTRO</t>
         </is>
       </c>
       <c r="D395" s="2" t="inlineStr">
         <is>
-          <t>14B-064_RF_TP_III_TV DO AMPARO - PRÓXIMO AO CETEP</t>
+          <t>14B-003_PTZ_PRACA FELIX GASPAR</t>
         </is>
       </c>
     </row>
@@ -9153,17 +9153,17 @@
       </c>
       <c r="B396" s="2" t="inlineStr">
         <is>
-          <t>CIRETRAN</t>
+          <t>UNIFACEMP - CENTRO UNIVERSITÁRIO DE CIÊNCIAS E EMPREENDEDORISMO</t>
         </is>
       </c>
       <c r="C396" s="2" t="inlineStr">
         <is>
-          <t>AV. ANTONIO CARLOS MAGALHAES, S/N - SÃO PAULO</t>
+          <t>RUA ANTONIO VEIGA ARGOLO, N 58 - CENTRO</t>
         </is>
       </c>
       <c r="D396" s="2" t="inlineStr">
         <is>
-          <t>14B-062_RF_TP_III_AV ANTONIO CARLOS NAGALHAES</t>
+          <t>14B-005_PTZ_RUA DOUTOR RENATO MACHADO</t>
         </is>
       </c>
     </row>
@@ -9175,17 +9175,17 @@
       </c>
       <c r="B397" s="2" t="inlineStr">
         <is>
-          <t>PRÉDIO ESCOLAR FLORENTINO FIRMINO DE ALMEIDA</t>
+          <t>UNIFACEMP - CENTRO UNIVERSITÁRIO DE CIÊNCIAS E EMPREENDEDORISMO</t>
         </is>
       </c>
       <c r="C397" s="2" t="inlineStr">
         <is>
-          <t>AV. ANTONIO CARLOS MAGALHÃES, S/N - SÃO PAULO</t>
+          <t>RUA ANTONIO VEIGA ARGOLO, N 58 - CENTRO</t>
         </is>
       </c>
       <c r="D397" s="2" t="inlineStr">
         <is>
-          <t>14B-054_LPR_AV HEITOR LIRIO DE MELO GRANNICK MARMORES STD CENTRO</t>
+          <t>14B-006_PTZ_R LANDULFO ALVES</t>
         </is>
       </c>
     </row>
@@ -9207,73 +9207,73 @@
       </c>
       <c r="D398" s="2" t="inlineStr">
         <is>
-          <t>14B-003_PTZ_PRACA FELIX GASPAR</t>
+          <t>14B-026_LPR_PRACA RENATO MACHADO STD MAGAZINE LUIZA</t>
         </is>
       </c>
     </row>
     <row r="399">
       <c r="A399" s="2" t="inlineStr">
         <is>
-          <t>SANTO ANTÔNIO DE JESUS</t>
+          <t>SANTO ESTEVÃO</t>
         </is>
       </c>
       <c r="B399" s="2" t="inlineStr">
         <is>
-          <t>UNIFACEMP - CENTRO UNIVERSITÁRIO DE CIÊNCIAS E EMPREENDEDORISMO</t>
+          <t>ESCOLA MUNICIPAL DOM PEDRO I</t>
         </is>
       </c>
       <c r="C399" s="2" t="inlineStr">
         <is>
-          <t>RUA ANTONIO VEIGA ARGOLO, N 58 - CENTRO</t>
+          <t>AV GETÚLIO VARGAS CENTRO</t>
         </is>
       </c>
       <c r="D399" s="2" t="inlineStr">
         <is>
-          <t>14B-005_PTZ_RUA DOUTOR RENATO MACHADO</t>
+          <t>57-007_LPR_AV GETULIO VAGAS AO LADO DO POSTO E HOTEL MARAMBAIA STD BR 116</t>
         </is>
       </c>
     </row>
     <row r="400">
       <c r="A400" s="2" t="inlineStr">
         <is>
-          <t>SANTO ANTÔNIO DE JESUS</t>
+          <t>SANTO ESTEVÃO</t>
         </is>
       </c>
       <c r="B400" s="2" t="inlineStr">
         <is>
-          <t>UNIFACEMP - CENTRO UNIVERSITÁRIO DE CIÊNCIAS E EMPREENDEDORISMO</t>
+          <t>ESCOLA MUNICIPAL MARIZELIA DE JESUS ROCHA LEAL</t>
         </is>
       </c>
       <c r="C400" s="2" t="inlineStr">
         <is>
-          <t>RUA ANTONIO VEIGA ARGOLO, N 58 - CENTRO</t>
+          <t>RUA MARECHAL FLORIANO PEIXOTO, S/N - CENTRO</t>
         </is>
       </c>
       <c r="D400" s="2" t="inlineStr">
         <is>
-          <t>14B-006_PTZ_R LANDULFO ALVES</t>
+          <t>57-002_PTZ_AV MARECHAL FLORIANO PEIXOTO EM FRENTE A ELIAS FERRAGENS</t>
         </is>
       </c>
     </row>
     <row r="401">
       <c r="A401" s="2" t="inlineStr">
         <is>
-          <t>SANTO ANTÔNIO DE JESUS</t>
+          <t>SANTO ESTEVÃO</t>
         </is>
       </c>
       <c r="B401" s="2" t="inlineStr">
         <is>
-          <t>UNIFACEMP - CENTRO UNIVERSITÁRIO DE CIÊNCIAS E EMPREENDEDORISMO</t>
+          <t>ESCOLA MUNICIPAL MONSENHOR JOSÉ WALDIR DE SOUZA</t>
         </is>
       </c>
       <c r="C401" s="2" t="inlineStr">
         <is>
-          <t>RUA ANTONIO VEIGA ARGOLO, N 58 - CENTRO</t>
+          <t>AVENIDA RIO BAHIA - TRIÂNGULO</t>
         </is>
       </c>
       <c r="D401" s="2" t="inlineStr">
         <is>
-          <t>14B-026_LPR_PRACA RENATO MACHADO STD MAGAZINE LUIZA</t>
+          <t>57-010_LPR_AV CASTRO ALVES EM FRENTE A CAIXA ECONOMICA</t>
         </is>
       </c>
     </row>
@@ -9285,149 +9285,149 @@
       </c>
       <c r="B402" s="2" t="inlineStr">
         <is>
-          <t>ESCOLA MUNICIPAL DOM PEDRO I</t>
+          <t>ESCOLA MUNICIPAL PROFESSOR JOSÉ AGNALDO BARRETO DE ALMEIDA</t>
         </is>
       </c>
       <c r="C402" s="2" t="inlineStr">
         <is>
-          <t>AV GETÚLIO VARGAS CENTRO</t>
+          <t>AVENIDA LUIZ VIANA   - CENTRO</t>
         </is>
       </c>
       <c r="D402" s="2" t="inlineStr">
         <is>
-          <t>57-007_LPR_AV GETULIO VAGAS AO LADO DO POSTO E HOTEL MARAMBAIA STD BR 116</t>
+          <t>57-008_LPR_AV LUIS VIANA FILHO - EM FRENTE A ESCOLA MUN JOSE AGNALDO STD CENTRO</t>
         </is>
       </c>
     </row>
     <row r="403">
       <c r="A403" s="2" t="inlineStr">
         <is>
-          <t>SANTO ESTEVÃO</t>
+          <t>SERRA DOURADA</t>
         </is>
       </c>
       <c r="B403" s="2" t="inlineStr">
         <is>
-          <t>ESCOLA MUNICIPAL MARIZELIA DE JESUS ROCHA LEAL</t>
+          <t>ESCOLA MINICÍPAL MONSENHOR FÉLIX</t>
         </is>
       </c>
       <c r="C403" s="2" t="inlineStr">
         <is>
-          <t>RUA MARECHAL FLORIANO PEIXOTO, S/N - CENTRO</t>
+          <t>PRACA FRANCISCO J. DE AQUINO - CENTRO</t>
         </is>
       </c>
       <c r="D403" s="2" t="inlineStr">
         <is>
-          <t>57-002_PTZ_AV MARECHAL FLORIANO PEIXOTO EM FRENTE A ELIAS FERRAGENS</t>
+          <t>30-030_PTZ_TRAVESSA DE ASSOCIACAO DE CAPOEIRA EM FRENTE AO FORUM</t>
         </is>
       </c>
     </row>
     <row r="404">
       <c r="A404" s="2" t="inlineStr">
         <is>
-          <t>SANTO ESTEVÃO</t>
+          <t>SERRA DOURADA</t>
         </is>
       </c>
       <c r="B404" s="2" t="inlineStr">
         <is>
-          <t>ESCOLA MUNICIPAL MONSENHOR JOSÉ WALDIR DE SOUZA</t>
+          <t>ESCOLA MINICÍPAL MONSENHOR FÉLIX</t>
         </is>
       </c>
       <c r="C404" s="2" t="inlineStr">
         <is>
-          <t>AVENIDA RIO BAHIA - TRIÂNGULO</t>
+          <t>PRACA FRANCISCO J. DE AQUINO - CENTRO</t>
         </is>
       </c>
       <c r="D404" s="2" t="inlineStr">
         <is>
-          <t>57-010_LPR_AV CASTRO ALVES EM FRENTE A CAIXA ECONOMICA</t>
+          <t>30-036_RF_TP_IV_AV MANSO CABRAL EM FRENTE AO HOSP MUN CARLITO C DA CUNHA</t>
         </is>
       </c>
     </row>
     <row r="405">
       <c r="A405" s="2" t="inlineStr">
         <is>
-          <t>SANTO ESTEVÃO</t>
+          <t>SERRA DOURADA</t>
         </is>
       </c>
       <c r="B405" s="2" t="inlineStr">
         <is>
-          <t>ESCOLA MUNICIPAL PROFESSOR JOSÉ AGNALDO BARRETO DE ALMEIDA</t>
+          <t>ESCOLA MUNICIPAL ELIEZER PEREIRA DA SILVA</t>
         </is>
       </c>
       <c r="C405" s="2" t="inlineStr">
         <is>
-          <t>AVENIDA LUIZ VIANA   - CENTRO</t>
+          <t>PRAÇA PEDRO JOSE DE AQUINO, S/N - CENTRO</t>
         </is>
       </c>
       <c r="D405" s="2" t="inlineStr">
         <is>
-          <t>57-008_LPR_AV LUIS VIANA FILHO - EM FRENTE A ESCOLA MUN JOSE AGNALDO STD CENTRO</t>
+          <t>30-029_PTZ_RUA ISIDORO BISPO NOGUEIRA</t>
         </is>
       </c>
     </row>
     <row r="406">
       <c r="A406" s="2" t="inlineStr">
         <is>
-          <t>SERRA DOURADA</t>
+          <t>SIMÕES FILHO</t>
         </is>
       </c>
       <c r="B406" s="2" t="inlineStr">
         <is>
-          <t>ESCOLA MINICÍPAL MONSENHOR FÉLIX</t>
+          <t>CENTRO COMUNITÁRIO NOSSA ESPERANÇA</t>
         </is>
       </c>
       <c r="C406" s="2" t="inlineStr">
         <is>
-          <t>PRACA FRANCISCO J. DE AQUINO - CENTRO</t>
+          <t>RUA NOVA ESPERANÇA S/N - PITANGA DE PALMARES</t>
         </is>
       </c>
       <c r="D406" s="2" t="inlineStr">
         <is>
-          <t>30-030_PTZ_TRAVESSA DE ASSOCIACAO DE CAPOEIRA EM FRENTE AO FORUM</t>
+          <t>SEAP-045_PTZ_ROD C DE TRAFEGO RUA M DOS S EM FRENTE UN SAUDE FAMILIA - RODOVIA CANAL DE TRAFEGO</t>
         </is>
       </c>
     </row>
     <row r="407">
       <c r="A407" s="2" t="inlineStr">
         <is>
-          <t>SERRA DOURADA</t>
+          <t>SIMÕES FILHO</t>
         </is>
       </c>
       <c r="B407" s="2" t="inlineStr">
         <is>
-          <t>ESCOLA MINICÍPAL MONSENHOR FÉLIX</t>
+          <t>CENTRO COMUNITÁRIO NOSSA IRMÃ DULCE</t>
         </is>
       </c>
       <c r="C407" s="2" t="inlineStr">
         <is>
-          <t>PRACA FRANCISCO J. DE AQUINO - CENTRO</t>
+          <t>BA 093 - SANTA ROSA</t>
         </is>
       </c>
       <c r="D407" s="2" t="inlineStr">
         <is>
-          <t>30-036_RF_TP_IV_AV MANSO CABRAL EM FRENTE AO HOSP MUN CARLITO C DA CUNHA</t>
+          <t>22-091_LPR_BA 093_STD_CAMACARI_ANTES DO POSTO BR COWBOY</t>
         </is>
       </c>
     </row>
     <row r="408">
       <c r="A408" s="2" t="inlineStr">
         <is>
-          <t>SERRA DOURADA</t>
+          <t>SIMÕES FILHO</t>
         </is>
       </c>
       <c r="B408" s="2" t="inlineStr">
         <is>
-          <t>ESCOLA MUNICIPAL ELIEZER PEREIRA DA SILVA</t>
+          <t>COLÉGIO ESTADUAL DE ARATU</t>
         </is>
       </c>
       <c r="C408" s="2" t="inlineStr">
         <is>
-          <t>PRAÇA PEDRO JOSE DE AQUINO, S/N - CENTRO</t>
+          <t>RUA COLÉGIO ESTADUAL DE ARATU, S/N, CIA I</t>
         </is>
       </c>
       <c r="D408" s="2" t="inlineStr">
         <is>
-          <t>30-029_PTZ_RUA ISIDORO BISPO NOGUEIRA</t>
+          <t>22-008_PTZ_R DR CARLOS CHAGAS QD 8 NUCLEO HAB RUBENS COSTA</t>
         </is>
       </c>
     </row>
@@ -9439,17 +9439,17 @@
       </c>
       <c r="B409" s="2" t="inlineStr">
         <is>
-          <t>CENTRO COMUNITÁRIO NOSSA ESPERANÇA</t>
+          <t>COLÉGIO ESTADUAL DE ARATU</t>
         </is>
       </c>
       <c r="C409" s="2" t="inlineStr">
         <is>
-          <t>RUA NOVA ESPERANÇA S/N - PITANGA DE PALMARES</t>
+          <t>RUA COLÉGIO ESTADUAL DE ARATU, S/N, CIA I</t>
         </is>
       </c>
       <c r="D409" s="2" t="inlineStr">
         <is>
-          <t>SEAP-045_PTZ_ROD C DE TRAFEGO RUA M DOS S EM FRENTE UN SAUDE FAMILIA - RODOVIA CANAL DE TRAFEGO</t>
+          <t>22-098_RF_TP_IV_AV ELMO SEREJO DE FARIAS PONTO DE ONIBUS EM FRENTE A UPA</t>
         </is>
       </c>
     </row>
@@ -9461,17 +9461,17 @@
       </c>
       <c r="B410" s="2" t="inlineStr">
         <is>
-          <t>CENTRO COMUNITÁRIO NOSSA IRMÃ DULCE</t>
+          <t>COLÉGIO ESTADUAL MANOEL DE JESUS</t>
         </is>
       </c>
       <c r="C410" s="2" t="inlineStr">
         <is>
-          <t>BA 093 - SANTA ROSA</t>
+          <t>PRAÇA DA BANDEIRA S/N</t>
         </is>
       </c>
       <c r="D410" s="2" t="inlineStr">
         <is>
-          <t>22-091_LPR_BA 093_STD_CAMACARI_ANTES DO POSTO BR COWBOY</t>
+          <t>22-016_PTZ_PRACA EMILIO FELIX</t>
         </is>
       </c>
     </row>
@@ -9483,17 +9483,17 @@
       </c>
       <c r="B411" s="2" t="inlineStr">
         <is>
-          <t>COLÉGIO ESTADUAL DE ARATU</t>
+          <t>ESCOLA ALBERTO SILVA</t>
         </is>
       </c>
       <c r="C411" s="2" t="inlineStr">
         <is>
-          <t>RUA COLÉGIO ESTADUAL DE ARATU, S/N, CIA I</t>
+          <t>PRAÇA SETE DE NOVEMBRO, S/N - CENTRO</t>
         </is>
       </c>
       <c r="D411" s="2" t="inlineStr">
         <is>
-          <t>22-008_PTZ_R DR CARLOS CHAGAS QD 8 NUCLEO HAB RUBENS COSTA</t>
+          <t>22-031_PTZ_AV ELMO SEREJO DE FARIAS - ROTATÓRIA EM FRENTE A MW AUTO PEÇAS</t>
         </is>
       </c>
     </row>
@@ -9505,17 +9505,17 @@
       </c>
       <c r="B412" s="2" t="inlineStr">
         <is>
-          <t>COLÉGIO ESTADUAL DE ARATU</t>
+          <t>ESCOLA BERLINDO MAMEDE</t>
         </is>
       </c>
       <c r="C412" s="2" t="inlineStr">
         <is>
-          <t>RUA COLÉGIO ESTADUAL DE ARATU, S/N, CIA I</t>
+          <t>RUA LOMANTO JUNIOR 71 - PONTO DE PARADA</t>
         </is>
       </c>
       <c r="D412" s="2" t="inlineStr">
         <is>
-          <t>22-098_RF_TP_IV_AV ELMO SEREJO DE FARIAS PONTO DE ONIBUS EM FRENTE A UPA</t>
+          <t>22-013_PTZ_PONTO PARADA R INOCENCIO ANTONIO DA ROCHA LOT MUNICIPAL</t>
         </is>
       </c>
     </row>
@@ -9527,17 +9527,17 @@
       </c>
       <c r="B413" s="2" t="inlineStr">
         <is>
-          <t>COLÉGIO ESTADUAL MANOEL DE JESUS</t>
+          <t>ESCOLA DOM FRANCISCO LEITE</t>
         </is>
       </c>
       <c r="C413" s="2" t="inlineStr">
         <is>
-          <t>PRAÇA DA BANDEIRA S/N</t>
+          <t>DISTRITO SANTA LUZIA - SANTA LUZIA</t>
         </is>
       </c>
       <c r="D413" s="2" t="inlineStr">
         <is>
-          <t>22-016_PTZ_PRACA EMILIO FELIX</t>
+          <t>22-015_PTZ_AV ALTAMIRANDO DE ARAUJO</t>
         </is>
       </c>
     </row>
@@ -9549,17 +9549,17 @@
       </c>
       <c r="B414" s="2" t="inlineStr">
         <is>
-          <t>ESCOLA ALBERTO SILVA</t>
+          <t>ESCOLA DOM FRANCISCO LEITE</t>
         </is>
       </c>
       <c r="C414" s="2" t="inlineStr">
         <is>
-          <t>PRAÇA SETE DE NOVEMBRO, S/N - CENTRO</t>
+          <t>DISTRITO SANTA LUZIA - SANTA LUZIA</t>
         </is>
       </c>
       <c r="D414" s="2" t="inlineStr">
         <is>
-          <t>22-031_PTZ_AV ELMO SEREJO DE FARIAS - ROTATÓRIA EM FRENTE A MW AUTO PEÇAS</t>
+          <t>22-018_PTZ_AV RUI BARBOSA</t>
         </is>
       </c>
     </row>
@@ -9571,17 +9571,17 @@
       </c>
       <c r="B415" s="2" t="inlineStr">
         <is>
-          <t>ESCOLA BERLINDO MAMEDE</t>
+          <t>ESCOLA DOM FRANCISCO LEITE</t>
         </is>
       </c>
       <c r="C415" s="2" t="inlineStr">
         <is>
-          <t>RUA LOMANTO JUNIOR 71 - PONTO DE PARADA</t>
+          <t>DISTRITO SANTA LUZIA - SANTA LUZIA</t>
         </is>
       </c>
       <c r="D415" s="2" t="inlineStr">
         <is>
-          <t>22-013_PTZ_PONTO PARADA R INOCENCIO ANTONIO DA ROCHA LOT MUNICIPAL</t>
+          <t>22-021_PTZ_AV A DE ARAUJO RAMOS CENTRO</t>
         </is>
       </c>
     </row>
@@ -9603,7 +9603,7 @@
       </c>
       <c r="D416" s="2" t="inlineStr">
         <is>
-          <t>22-015_PTZ_AV ALTAMIRANDO DE ARAUJO</t>
+          <t>22-068_RF_TP_IV_AVENIDA RUI BARBOSA_EM FRENTE_CENTRO COMERCIAL WALTER GOMES</t>
         </is>
       </c>
     </row>
@@ -9625,7 +9625,7 @@
       </c>
       <c r="D417" s="2" t="inlineStr">
         <is>
-          <t>22-018_PTZ_AV RUI BARBOSA</t>
+          <t>22-097_RF_TP_III_AV ALTAMIRANDO DE ARAUJO RAMOS_EM FRENTE AO BANCO ITAU</t>
         </is>
       </c>
     </row>
@@ -9637,17 +9637,17 @@
       </c>
       <c r="B418" s="2" t="inlineStr">
         <is>
-          <t>ESCOLA DOM FRANCISCO LEITE</t>
+          <t>ESCOLA MUNICIPAL ANTÔNIA SOUZA DE SANTANA</t>
         </is>
       </c>
       <c r="C418" s="2" t="inlineStr">
         <is>
-          <t>DISTRITO SANTA LUZIA - SANTA LUZIA</t>
+          <t>AVENIDA POTY, S/N - COTEGIPE</t>
         </is>
       </c>
       <c r="D418" s="2" t="inlineStr">
         <is>
-          <t>22-021_PTZ_AV A DE ARAUJO RAMOS CENTRO</t>
+          <t>22-015_PTZ_AV ALTAMIRANDO DE ARAUJO</t>
         </is>
       </c>
     </row>
@@ -9659,17 +9659,17 @@
       </c>
       <c r="B419" s="2" t="inlineStr">
         <is>
-          <t>ESCOLA DOM FRANCISCO LEITE</t>
+          <t>ESCOLA MUNICIPAL ANTÔNIA SOUZA DE SANTANA</t>
         </is>
       </c>
       <c r="C419" s="2" t="inlineStr">
         <is>
-          <t>DISTRITO SANTA LUZIA - SANTA LUZIA</t>
+          <t>AVENIDA POTY, S/N - COTEGIPE</t>
         </is>
       </c>
       <c r="D419" s="2" t="inlineStr">
         <is>
-          <t>22-068_RF_TP_IV_AVENIDA RUI BARBOSA_EM FRENTE_CENTRO COMERCIAL WALTER GOMES</t>
+          <t>22-018_PTZ_AV RUI BARBOSA</t>
         </is>
       </c>
     </row>
@@ -9681,17 +9681,17 @@
       </c>
       <c r="B420" s="2" t="inlineStr">
         <is>
-          <t>ESCOLA DOM FRANCISCO LEITE</t>
+          <t>ESCOLA MUNICIPAL ANTÔNIA SOUZA DE SANTANA</t>
         </is>
       </c>
       <c r="C420" s="2" t="inlineStr">
         <is>
-          <t>DISTRITO SANTA LUZIA - SANTA LUZIA</t>
+          <t>AVENIDA POTY, S/N - COTEGIPE</t>
         </is>
       </c>
       <c r="D420" s="2" t="inlineStr">
         <is>
-          <t>22-097_RF_TP_III_AV ALTAMIRANDO DE ARAUJO RAMOS_EM FRENTE AO BANCO ITAU</t>
+          <t>22-021_PTZ_AV A DE ARAUJO RAMOS CENTRO</t>
         </is>
       </c>
     </row>
@@ -9713,7 +9713,7 @@
       </c>
       <c r="D421" s="2" t="inlineStr">
         <is>
-          <t>22-015_PTZ_AV ALTAMIRANDO DE ARAUJO</t>
+          <t>22-068_RF_TP_IV_AVENIDA RUI BARBOSA_EM FRENTE_CENTRO COMERCIAL WALTER GOMES</t>
         </is>
       </c>
     </row>
@@ -9735,7 +9735,7 @@
       </c>
       <c r="D422" s="2" t="inlineStr">
         <is>
-          <t>22-018_PTZ_AV RUI BARBOSA</t>
+          <t>22-097_RF_TP_III_AV ALTAMIRANDO DE ARAUJO RAMOS_EM FRENTE AO BANCO ITAU</t>
         </is>
       </c>
     </row>
@@ -9747,17 +9747,17 @@
       </c>
       <c r="B423" s="2" t="inlineStr">
         <is>
-          <t>ESCOLA MUNICIPAL ANTÔNIA SOUZA DE SANTANA</t>
+          <t>ESCOLA MUNICIPAL IDALIA CLEMENTE BRAGA BESTOSO</t>
         </is>
       </c>
       <c r="C423" s="2" t="inlineStr">
         <is>
-          <t>AVENIDA POTY, S/N - COTEGIPE</t>
+          <t>CONJUNTO ILHA DE SÃO JOÃO - ILHA DE SÃO JOÃO</t>
         </is>
       </c>
       <c r="D423" s="2" t="inlineStr">
         <is>
-          <t>22-021_PTZ_AV A DE ARAUJO RAMOS CENTRO</t>
+          <t>22-001_PTZ_RUA ILHA CJ ILHA SAO JOAO</t>
         </is>
       </c>
     </row>
@@ -9769,17 +9769,17 @@
       </c>
       <c r="B424" s="2" t="inlineStr">
         <is>
-          <t>ESCOLA MUNICIPAL ANTÔNIA SOUZA DE SANTANA</t>
+          <t>ESCOLA REITOR MIGUEL CALMON</t>
         </is>
       </c>
       <c r="C424" s="2" t="inlineStr">
         <is>
-          <t>AVENIDA POTY, S/N - COTEGIPE</t>
+          <t>RUA GENERAL LABATUT, S/N - PONTO DE PARADA</t>
         </is>
       </c>
       <c r="D424" s="2" t="inlineStr">
         <is>
-          <t>22-068_RF_TP_IV_AVENIDA RUI BARBOSA_EM FRENTE_CENTRO COMERCIAL WALTER GOMES</t>
+          <t>22-012_PTZ_RUA FRANCISCO COPIRUNGA CONJ HAB CIA II</t>
         </is>
       </c>
     </row>
@@ -9791,17 +9791,17 @@
       </c>
       <c r="B425" s="2" t="inlineStr">
         <is>
-          <t>ESCOLA MUNICIPAL ANTÔNIA SOUZA DE SANTANA</t>
+          <t>ESCOLA REITOR MIGUEL CALMON</t>
         </is>
       </c>
       <c r="C425" s="2" t="inlineStr">
         <is>
-          <t>AVENIDA POTY, S/N - COTEGIPE</t>
+          <t>RUA GENERAL LABATUT, S/N - PONTO DE PARADA</t>
         </is>
       </c>
       <c r="D425" s="2" t="inlineStr">
         <is>
-          <t>22-097_RF_TP_III_AV ALTAMIRANDO DE ARAUJO RAMOS_EM FRENTE AO BANCO ITAU</t>
+          <t>22-055_RF_TP_III_R MAL HERMES DA FONSECA_PROX_22CIPM</t>
         </is>
       </c>
     </row>
@@ -9813,17 +9813,17 @@
       </c>
       <c r="B426" s="2" t="inlineStr">
         <is>
-          <t>ESCOLA MUNICIPAL IDALIA CLEMENTE BRAGA BESTOSO</t>
+          <t>ESCOLA VEREADOR JOÃO DE OLIVEIRA CAMPOS</t>
         </is>
       </c>
       <c r="C426" s="2" t="inlineStr">
         <is>
-          <t>CONJUNTO ILHA DE SÃO JOÃO - ILHA DE SÃO JOÃO</t>
+          <t>AV ENGENHEIRO ELMO SEREJO DE FARIAS S/N - CIA I</t>
         </is>
       </c>
       <c r="D426" s="2" t="inlineStr">
         <is>
-          <t>22-001_PTZ_RUA ILHA CJ ILHA SAO JOAO</t>
+          <t>22-063_RF_TP_IV_R OSVALDO CRUZ_EM FRENTE A UPA SIMÕES FILHO</t>
         </is>
       </c>
     </row>
@@ -9835,83 +9835,83 @@
       </c>
       <c r="B427" s="2" t="inlineStr">
         <is>
-          <t>ESCOLA REITOR MIGUEL CALMON</t>
+          <t>ESCOLA VEREADOR JOÃO DE OLIVEIRA CAMPOS</t>
         </is>
       </c>
       <c r="C427" s="2" t="inlineStr">
         <is>
-          <t>RUA GENERAL LABATUT, S/N - PONTO DE PARADA</t>
+          <t>AV ENGENHEIRO ELMO SEREJO DE FARIAS S/N - CIA I</t>
         </is>
       </c>
       <c r="D427" s="2" t="inlineStr">
         <is>
-          <t>22-012_PTZ_RUA FRANCISCO COPIRUNGA CONJ HAB CIA II</t>
+          <t>22-098_RF_TP_IV_AV ELMO SEREJO DE FARIAS PONTO DE ONIBUS EM FRENTE A UPA</t>
         </is>
       </c>
     </row>
     <row r="428">
       <c r="A428" s="2" t="inlineStr">
         <is>
-          <t>SIMÕES FILHO</t>
+          <t>SÃO FRANCISCO DO CONDE</t>
         </is>
       </c>
       <c r="B428" s="2" t="inlineStr">
         <is>
-          <t>ESCOLA REITOR MIGUEL CALMON</t>
+          <t>ESCOLA ESTADUAL ANA JUNQUEIRA AYRES TOURINHO</t>
         </is>
       </c>
       <c r="C428" s="2" t="inlineStr">
         <is>
-          <t>RUA GENERAL LABATUT, S/N - PONTO DE PARADA</t>
+          <t>RUA DO ASFALTO, S/N - POVOADO CAÍPE</t>
         </is>
       </c>
       <c r="D428" s="2" t="inlineStr">
         <is>
-          <t>22-055_RF_TP_III_R MAL HERMES DA FONSECA_PROX_22CIPM</t>
+          <t>10-167_PTZ_AV M B R EM FRENTE ESCOLA M INTEGRAL DE CAIPE</t>
         </is>
       </c>
     </row>
     <row r="429">
       <c r="A429" s="2" t="inlineStr">
         <is>
-          <t>SIMÕES FILHO</t>
+          <t>SÃO FRANCISCO DO CONDE</t>
         </is>
       </c>
       <c r="B429" s="2" t="inlineStr">
         <is>
-          <t>ESCOLA VEREADOR JOÃO DE OLIVEIRA CAMPOS</t>
+          <t>ESCOLA MUNICIPAL LÍCIA PINHO</t>
         </is>
       </c>
       <c r="C429" s="2" t="inlineStr">
         <is>
-          <t>AV ENGENHEIRO ELMO SEREJO DE FARIAS S/N - CIA I</t>
+          <t>RUA ESPÍRITO SANTO, S/N - CENTRO</t>
         </is>
       </c>
       <c r="D429" s="2" t="inlineStr">
         <is>
-          <t>22-063_RF_TP_IV_R OSVALDO CRUZ_EM FRENTE A UPA SIMÕES FILHO</t>
+          <t>10-056_PTZ_RUA DO ASFALTO</t>
         </is>
       </c>
     </row>
     <row r="430">
       <c r="A430" s="2" t="inlineStr">
         <is>
-          <t>SIMÕES FILHO</t>
+          <t>SÃO FRANCISCO DO CONDE</t>
         </is>
       </c>
       <c r="B430" s="2" t="inlineStr">
         <is>
-          <t>ESCOLA VEREADOR JOÃO DE OLIVEIRA CAMPOS</t>
+          <t>ESCOLA RURAL</t>
         </is>
       </c>
       <c r="C430" s="2" t="inlineStr">
         <is>
-          <t>AV ENGENHEIRO ELMO SEREJO DE FARIAS S/N - CIA I</t>
+          <t>PRAÇA ALZIRA SANTANA CRUZ, S/N - POVOADO PARAMIRIM</t>
         </is>
       </c>
       <c r="D430" s="2" t="inlineStr">
         <is>
-          <t>22-098_RF_TP_IV_AV ELMO SEREJO DE FARIAS PONTO DE ONIBUS EM FRENTE A UPA</t>
+          <t>10-042_PTZ_MATARIPE SAO FRANCISCO DO CONDE</t>
         </is>
       </c>
     </row>
@@ -9923,17 +9923,17 @@
       </c>
       <c r="B431" s="2" t="inlineStr">
         <is>
-          <t>ESCOLA ESTADUAL ANA JUNQUEIRA AYRES TOURINHO</t>
+          <t>FREI ELISEU EISMANN</t>
         </is>
       </c>
       <c r="C431" s="2" t="inlineStr">
         <is>
-          <t>RUA DO ASFALTO, S/N - POVOADO CAÍPE</t>
+          <t>RUA FREI MIGUEL, S/N - CENTRO</t>
         </is>
       </c>
       <c r="D431" s="2" t="inlineStr">
         <is>
-          <t>10-167_PTZ_AV M B R EM FRENTE ESCOLA M INTEGRAL DE CAIPE</t>
+          <t>10-047_PTZ_ RUA FREI MIGUEL CENTRO</t>
         </is>
       </c>
     </row>
@@ -9945,17 +9945,17 @@
       </c>
       <c r="B432" s="2" t="inlineStr">
         <is>
-          <t>ESCOLA MUNICIPAL LÍCIA PINHO</t>
+          <t>FREI ELISEU EISMANN</t>
         </is>
       </c>
       <c r="C432" s="2" t="inlineStr">
         <is>
-          <t>RUA ESPÍRITO SANTO, S/N - CENTRO</t>
+          <t>RUA FREI MIGUEL, S/N - CENTRO</t>
         </is>
       </c>
       <c r="D432" s="2" t="inlineStr">
         <is>
-          <t>10-056_PTZ_RUA DO ASFALTO</t>
+          <t>10-048_PTZ_RUA FREI MIGUEL</t>
         </is>
       </c>
     </row>
@@ -9967,17 +9967,17 @@
       </c>
       <c r="B433" s="2" t="inlineStr">
         <is>
-          <t>ESCOLA RURAL</t>
+          <t>FREI ELISEU EISMANN</t>
         </is>
       </c>
       <c r="C433" s="2" t="inlineStr">
         <is>
-          <t>PRAÇA ALZIRA SANTANA CRUZ, S/N - POVOADO PARAMIRIM</t>
+          <t>RUA FREI MIGUEL, S/N - CENTRO</t>
         </is>
       </c>
       <c r="D433" s="2" t="inlineStr">
         <is>
-          <t>10-042_PTZ_MATARIPE SAO FRANCISCO DO CONDE</t>
+          <t>10-163_PTZ_R CASTRO ALVES 15 EM FRENTE A DAY TECH</t>
         </is>
       </c>
     </row>
@@ -9989,83 +9989,83 @@
       </c>
       <c r="B434" s="2" t="inlineStr">
         <is>
-          <t>FREI ELISEU EISMANN</t>
+          <t>GINÁSIO LUIS VIANA NETO</t>
         </is>
       </c>
       <c r="C434" s="2" t="inlineStr">
         <is>
-          <t>RUA FREI MIGUEL, S/N - CENTRO</t>
+          <t>PRAÇA DA BANDEIRA - CENTRO</t>
         </is>
       </c>
       <c r="D434" s="2" t="inlineStr">
         <is>
-          <t>10-047_PTZ_ RUA FREI MIGUEL CENTRO</t>
+          <t>10-054_PTZ JOAO FLORENCIO GOMES PRACA EM FRENTE AO CRAS</t>
         </is>
       </c>
     </row>
     <row r="435">
       <c r="A435" s="2" t="inlineStr">
         <is>
-          <t>SÃO FRANCISCO DO CONDE</t>
+          <t>SÃO MIGUEL DAS MATAS</t>
         </is>
       </c>
       <c r="B435" s="2" t="inlineStr">
         <is>
-          <t>FREI ELISEU EISMANN</t>
+          <t>COLÉGIO ESTADUAL ALDEMIRO VILAS BOAS</t>
         </is>
       </c>
       <c r="C435" s="2" t="inlineStr">
         <is>
-          <t>RUA FREI MIGUEL, S/N - CENTRO</t>
+          <t>RUA RUI BARBOSA, S/N - CENTRO</t>
         </is>
       </c>
       <c r="D435" s="2" t="inlineStr">
         <is>
-          <t>10-048_PTZ_RUA FREI MIGUEL</t>
+          <t>99-020_LPR_RUA SAO ROQUE COL EST ALMERINDO VILAS BOAS STD CENTRO</t>
         </is>
       </c>
     </row>
     <row r="436">
       <c r="A436" s="2" t="inlineStr">
         <is>
-          <t>SÃO FRANCISCO DO CONDE</t>
+          <t>SÃO MIGUEL DAS MATAS</t>
         </is>
       </c>
       <c r="B436" s="2" t="inlineStr">
         <is>
-          <t>FREI ELISEU EISMANN</t>
+          <t>COLÉGIO MUNICIPAL PROFESSORA MARINEIDE REGINA SANTOS SOUSA</t>
         </is>
       </c>
       <c r="C436" s="2" t="inlineStr">
         <is>
-          <t>RUA FREI MIGUEL, S/N - CENTRO</t>
+          <t>RUA CÔNEGO POMPILIO, S/N - CENTRO</t>
         </is>
       </c>
       <c r="D436" s="2" t="inlineStr">
         <is>
-          <t>10-163_PTZ_R CASTRO ALVES 15 EM FRENTE A DAY TECH</t>
+          <t>99-019_PTZ_PRACA MARIA MADALENA EM FRENTE AO COLEGIO JOSE MARCELINO</t>
         </is>
       </c>
     </row>
     <row r="437">
       <c r="A437" s="2" t="inlineStr">
         <is>
-          <t>SÃO FRANCISCO DO CONDE</t>
+          <t>SÃO MIGUEL DAS MATAS</t>
         </is>
       </c>
       <c r="B437" s="2" t="inlineStr">
         <is>
-          <t>GINÁSIO LUIS VIANA NETO</t>
+          <t>COLÉGIO MUNICIPAL PROFESSORA MARINEIDE REGINA SANTOS SOUSA</t>
         </is>
       </c>
       <c r="C437" s="2" t="inlineStr">
         <is>
-          <t>PRAÇA DA BANDEIRA - CENTRO</t>
+          <t>RUA CÔNEGO POMPILIO, S/N - CENTRO</t>
         </is>
       </c>
       <c r="D437" s="2" t="inlineStr">
         <is>
-          <t>10-054_PTZ JOAO FLORENCIO GOMES PRACA EM FRENTE AO CRAS</t>
+          <t>99-023_RF_TP_IV_RUA CONEGO POMPILIO EM FRENTE AO BANCO DO BRASIL</t>
         </is>
       </c>
     </row>
@@ -10077,7 +10077,7 @@
       </c>
       <c r="B438" s="2" t="inlineStr">
         <is>
-          <t>COLÉGIO ESTADUAL ALDEMIRO VILAS BOAS</t>
+          <t>ESCOLA MUNICIPAL LOMANTO JÚNIOR</t>
         </is>
       </c>
       <c r="C438" s="2" t="inlineStr">
@@ -10094,66 +10094,66 @@
     <row r="439">
       <c r="A439" s="2" t="inlineStr">
         <is>
-          <t>SÃO MIGUEL DAS MATAS</t>
+          <t>SÃO SEBASTIÃO DO PASSÉ</t>
         </is>
       </c>
       <c r="B439" s="2" t="inlineStr">
         <is>
-          <t>COLÉGIO MUNICIPAL PROFESSORA MARINEIDE REGINA SANTOS SOUSA</t>
+          <t>ESCOLA MUNICIPAL DR JOÃO PAIM</t>
         </is>
       </c>
       <c r="C439" s="2" t="inlineStr">
         <is>
-          <t>RUA CÔNEGO POMPILIO, S/N - CENTRO</t>
+          <t>RUA EUTIQUIO DE LIMA, 155 - SAO ROQUE - CENTRO</t>
         </is>
       </c>
       <c r="D439" s="2" t="inlineStr">
         <is>
-          <t>99-019_PTZ_PRACA MARIA MADALENA EM FRENTE AO COLEGIO JOSE MARCELINO</t>
+          <t>10-005_PTZ_R CONEGO EUTIQUIO DE LIMA</t>
         </is>
       </c>
     </row>
     <row r="440">
       <c r="A440" s="2" t="inlineStr">
         <is>
-          <t>SÃO MIGUEL DAS MATAS</t>
+          <t>SÃO SEBASTIÃO DO PASSÉ</t>
         </is>
       </c>
       <c r="B440" s="2" t="inlineStr">
         <is>
-          <t>COLÉGIO MUNICIPAL PROFESSORA MARINEIDE REGINA SANTOS SOUSA</t>
+          <t>ESCOLA MUNICIPAL RÔMULO GALVÃO</t>
         </is>
       </c>
       <c r="C440" s="2" t="inlineStr">
         <is>
-          <t>RUA CÔNEGO POMPILIO, S/N - CENTRO</t>
+          <t>AV. ERNANE DE OLIVEIRA ROCHA, SN, PENAO - PENÃO</t>
         </is>
       </c>
       <c r="D440" s="2" t="inlineStr">
         <is>
-          <t>99-023_RF_TP_IV_RUA CONEGO POMPILIO EM FRENTE AO BANCO DO BRASIL</t>
+          <t>10-091_LPR_BR420 - EM FRENTE AO ESTADIO ANTONIO PENA- STD POSTO PETROBRAS</t>
         </is>
       </c>
     </row>
     <row r="441">
       <c r="A441" s="2" t="inlineStr">
         <is>
-          <t>SÃO MIGUEL DAS MATAS</t>
+          <t>SÃO SEBASTIÃO DO PASSÉ</t>
         </is>
       </c>
       <c r="B441" s="2" t="inlineStr">
         <is>
-          <t>ESCOLA MUNICIPAL LOMANTO JÚNIOR</t>
+          <t>ESCOLA MUNICIPAL RÔMULO GALVÃO</t>
         </is>
       </c>
       <c r="C441" s="2" t="inlineStr">
         <is>
-          <t>RUA RUI BARBOSA, S/N - CENTRO</t>
+          <t>AV. ERNANE DE OLIVEIRA ROCHA, SN, PENAO - PENÃO</t>
         </is>
       </c>
       <c r="D441" s="2" t="inlineStr">
         <is>
-          <t>99-020_LPR_RUA SAO ROQUE COL EST ALMERINDO VILAS BOAS STD CENTRO</t>
+          <t>10-129 PTZ R SERGIPE AO LADO IGREJA ASSEMBLEIA DE DEUS</t>
         </is>
       </c>
     </row>
@@ -10165,17 +10165,17 @@
       </c>
       <c r="B442" s="2" t="inlineStr">
         <is>
-          <t>ESCOLA MUNICIPAL DR JOÃO PAIM</t>
+          <t>ESCOLA MUNICIPAL RÔMULO GALVÃO</t>
         </is>
       </c>
       <c r="C442" s="2" t="inlineStr">
         <is>
-          <t>RUA EUTIQUIO DE LIMA, 155 - SAO ROQUE - CENTRO</t>
+          <t>AV. ERNANE DE OLIVEIRA ROCHA, SN, PENAO - PENÃO</t>
         </is>
       </c>
       <c r="D442" s="2" t="inlineStr">
         <is>
-          <t>10-005_PTZ_R CONEGO EUTIQUIO DE LIMA</t>
+          <t>10-172_PTZ_AV ERNANI DE OLIVEIRA ROCHA EM FRENTE AO ESTADIO MUNICIPAL ANTONIO PENA</t>
         </is>
       </c>
     </row>
@@ -10187,83 +10187,83 @@
       </c>
       <c r="B443" s="2" t="inlineStr">
         <is>
-          <t>ESCOLA MUNICIPAL RÔMULO GALVÃO</t>
+          <t>ESCOLA PROFESSORA LINDAURA MONTEIRO CÂMARA</t>
         </is>
       </c>
       <c r="C443" s="2" t="inlineStr">
         <is>
-          <t>AV. ERNANE DE OLIVEIRA ROCHA, SN, PENAO - PENÃO</t>
+          <t>RUA JOSÉ GONÇALVES, N 20 - CENTRO</t>
         </is>
       </c>
       <c r="D443" s="2" t="inlineStr">
         <is>
-          <t>10-091_LPR_BR420 - EM FRENTE AO ESTADIO ANTONIO PENA- STD POSTO PETROBRAS</t>
+          <t>10-102_RF_TP_III_BA 512_TERMINAL RODOVIARIO DE S SEBASTIAO DO PASSE</t>
         </is>
       </c>
     </row>
     <row r="444">
       <c r="A444" s="2" t="inlineStr">
         <is>
-          <t>SÃO SEBASTIÃO DO PASSÉ</t>
+          <t>TEIXEIRA DE FREITAS</t>
         </is>
       </c>
       <c r="B444" s="2" t="inlineStr">
         <is>
-          <t>ESCOLA MUNICIPAL RÔMULO GALVÃO</t>
+          <t>CONJUNTO PENAL DE TEIXEIRA DE FREITAS</t>
         </is>
       </c>
       <c r="C444" s="2" t="inlineStr">
         <is>
-          <t>AV. ERNANE DE OLIVEIRA ROCHA, SN, PENAO - PENÃO</t>
+          <t>CONJUNTO PENAL DE TEIXEIRA DE FREITAS</t>
         </is>
       </c>
       <c r="D444" s="2" t="inlineStr">
         <is>
-          <t>10-129 PTZ R SERGIPE AO LADO IGREJA ASSEMBLEIA DE DEUS</t>
+          <t>SEAP-I-080_PTZ_R NOVA VENECIA EM FRENTE AO PRESIDIO</t>
         </is>
       </c>
     </row>
     <row r="445">
       <c r="A445" s="2" t="inlineStr">
         <is>
-          <t>SÃO SEBASTIÃO DO PASSÉ</t>
+          <t>TEIXEIRA DE FREITAS</t>
         </is>
       </c>
       <c r="B445" s="2" t="inlineStr">
         <is>
-          <t>ESCOLA MUNICIPAL RÔMULO GALVÃO</t>
+          <t>CONJUNTO PENAL DE TEIXEIRA DE FREITAS</t>
         </is>
       </c>
       <c r="C445" s="2" t="inlineStr">
         <is>
-          <t>AV. ERNANE DE OLIVEIRA ROCHA, SN, PENAO - PENÃO</t>
+          <t>CONJUNTO PENAL DE TEIXEIRA DE FREITAS</t>
         </is>
       </c>
       <c r="D445" s="2" t="inlineStr">
         <is>
-          <t>10-172_PTZ_AV ERNANI DE OLIVEIRA ROCHA EM FRENTE AO ESTADIO MUNICIPAL ANTONIO PENA</t>
+          <t>SEAP-I-081_PTZ_R VINTE E CINCO AO LADO DO PRESIDIO</t>
         </is>
       </c>
     </row>
     <row r="446">
       <c r="A446" s="2" t="inlineStr">
         <is>
-          <t>SÃO SEBASTIÃO DO PASSÉ</t>
+          <t>TEIXEIRA DE FREITAS</t>
         </is>
       </c>
       <c r="B446" s="2" t="inlineStr">
         <is>
-          <t>ESCOLA PROFESSORA LINDAURA MONTEIRO CÂMARA</t>
+          <t>CONJUNTO PENAL DE TEIXEIRA DE FREITAS</t>
         </is>
       </c>
       <c r="C446" s="2" t="inlineStr">
         <is>
-          <t>RUA JOSÉ GONÇALVES, N 20 - CENTRO</t>
+          <t>CONJUNTO PENAL DE TEIXEIRA DE FREITAS</t>
         </is>
       </c>
       <c r="D446" s="2" t="inlineStr">
         <is>
-          <t>10-102_RF_TP_III_BA 512_TERMINAL RODOVIARIO DE S SEBASTIAO DO PASSE</t>
+          <t>SEAP-I-117_LPR_R NOVA VENECIA EM FRENTE A ENTRADA DO PRESIDIO STD PRESIDIO</t>
         </is>
       </c>
     </row>
@@ -10275,149 +10275,149 @@
       </c>
       <c r="B447" s="2" t="inlineStr">
         <is>
-          <t>CONJUNTO PENAL DE TEIXEIRA DE FREITAS</t>
+          <t>UNIVERSIDADE DO ESTADO DA BAHIA - UNEB</t>
         </is>
       </c>
       <c r="C447" s="2" t="inlineStr">
         <is>
-          <t>CONJUNTO PENAL DE TEIXEIRA DE FREITAS</t>
+          <t>AVENIDA KAIKAN, S/N - KAIKAN</t>
         </is>
       </c>
       <c r="D447" s="2" t="inlineStr">
         <is>
-          <t>SEAP-I-080_PTZ_R NOVA VENECIA EM FRENTE AO PRESIDIO</t>
+          <t>87-040_LPR_AVENIDA KAIKAN AO LADO DO CAMPOS BAR E A UNEB STD PRESIDIO</t>
         </is>
       </c>
     </row>
     <row r="448">
       <c r="A448" s="2" t="inlineStr">
         <is>
-          <t>TEIXEIRA DE FREITAS</t>
+          <t>UBATÃ</t>
         </is>
       </c>
       <c r="B448" s="2" t="inlineStr">
         <is>
-          <t>CONJUNTO PENAL DE TEIXEIRA DE FREITAS</t>
+          <t>COLEGIO ESTADUAL DE UBATA - CEU</t>
         </is>
       </c>
       <c r="C448" s="2" t="inlineStr">
         <is>
-          <t>CONJUNTO PENAL DE TEIXEIRA DE FREITAS</t>
+          <t>AVENIDA LANDULFO ALVES - CENTRO</t>
         </is>
       </c>
       <c r="D448" s="2" t="inlineStr">
         <is>
-          <t>SEAP-I-081_PTZ_R VINTE E CINCO AO LADO DO PRESIDIO</t>
+          <t>61-008_RF_TP_IV_AVENIDA LANDULFO ALVES EM FRENTE AO COL EST DE UBATA</t>
         </is>
       </c>
     </row>
     <row r="449">
       <c r="A449" s="2" t="inlineStr">
         <is>
-          <t>TEIXEIRA DE FREITAS</t>
+          <t>UBAÍRA</t>
         </is>
       </c>
       <c r="B449" s="2" t="inlineStr">
         <is>
-          <t>CONJUNTO PENAL DE TEIXEIRA DE FREITAS</t>
+          <t>ESCOLA MUNICIPAL RODRIGO DE SOUZA</t>
         </is>
       </c>
       <c r="C449" s="2" t="inlineStr">
         <is>
-          <t>CONJUNTO PENAL DE TEIXEIRA DE FREITAS</t>
+          <t>PRACA DOS TRES PODERES - CENTRO</t>
         </is>
       </c>
       <c r="D449" s="2" t="inlineStr">
         <is>
-          <t>SEAP-I-117_LPR_R NOVA VENECIA EM FRENTE A ENTRADA DO PRESIDIO STD PRESIDIO</t>
+          <t>14B-041_PTZ_RUA FERNANDES BARRETOS AO LADO DA PREFEITURA</t>
         </is>
       </c>
     </row>
     <row r="450">
       <c r="A450" s="2" t="inlineStr">
         <is>
-          <t>TEIXEIRA DE FREITAS</t>
+          <t>UBAÍRA</t>
         </is>
       </c>
       <c r="B450" s="2" t="inlineStr">
         <is>
-          <t>UNIVERSIDADE DO ESTADO DA BAHIA - UNEB</t>
+          <t>GRUPO ESCOLAR ANISIO TEIXEIRA</t>
         </is>
       </c>
       <c r="C450" s="2" t="inlineStr">
         <is>
-          <t>AVENIDA KAIKAN, S/N - KAIKAN</t>
+          <t>PRACA DOS TRES PODERES - CENTRO</t>
         </is>
       </c>
       <c r="D450" s="2" t="inlineStr">
         <is>
-          <t>87-040_LPR_AVENIDA KAIKAN AO LADO DO CAMPOS BAR E A UNEB STD PRESIDIO</t>
+          <t>14B-041_PTZ_RUA FERNANDES BARRETOS AO LADO DA PREFEITURA</t>
         </is>
       </c>
     </row>
     <row r="451">
       <c r="A451" s="2" t="inlineStr">
         <is>
-          <t>UBATÃ</t>
+          <t>VALENÇA</t>
         </is>
       </c>
       <c r="B451" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO ESTADUAL DE UBATA - CEU</t>
+          <t>CENTRO ESTADUAL EDUCAÇÃO PROF E SAÚDE DO L BAIANO-CEEP(ANTIGO COESVA)</t>
         </is>
       </c>
       <c r="C451" s="2" t="inlineStr">
         <is>
-          <t>AVENIDA LANDULFO ALVES - CENTRO</t>
+          <t>RUA FLORESTAL, 01 - BOLÍVIA</t>
         </is>
       </c>
       <c r="D451" s="2" t="inlineStr">
         <is>
-          <t>61-008_RF_TP_IV_AVENIDA LANDULFO ALVES EM FRENTE AO COL EST DE UBATA</t>
+          <t>33-039_PTZ_RUA DIRETA DA BOLIVIA_PRX DA IGREJA</t>
         </is>
       </c>
     </row>
     <row r="452">
       <c r="A452" s="2" t="inlineStr">
         <is>
-          <t>UBAÍRA</t>
+          <t>VALENÇA</t>
         </is>
       </c>
       <c r="B452" s="2" t="inlineStr">
         <is>
-          <t>ESCOLA MUNICIPAL RODRIGO DE SOUZA</t>
+          <t>COLÉGIO PERSPECTIVA</t>
         </is>
       </c>
       <c r="C452" s="2" t="inlineStr">
         <is>
-          <t>PRACA DOS TRES PODERES - CENTRO</t>
+          <t>PRAÇA CONSELHEIRO BALTAZAR, 138, TRIANA - CENTRO</t>
         </is>
       </c>
       <c r="D452" s="2" t="inlineStr">
         <is>
-          <t>14B-041_PTZ_RUA FERNANDES BARRETOS AO LADO DA PREFEITURA</t>
+          <t>33-022_RF_TERMINAL RODOVIARIO DE VALENCA</t>
         </is>
       </c>
     </row>
     <row r="453">
       <c r="A453" s="2" t="inlineStr">
         <is>
-          <t>UBAÍRA</t>
+          <t>VALENÇA</t>
         </is>
       </c>
       <c r="B453" s="2" t="inlineStr">
         <is>
-          <t>GRUPO ESCOLAR ANISIO TEIXEIRA</t>
+          <t>COLÉGIO PERSPECTIVA</t>
         </is>
       </c>
       <c r="C453" s="2" t="inlineStr">
         <is>
-          <t>PRACA DOS TRES PODERES - CENTRO</t>
+          <t>PRAÇA CONSELHEIRO BALTAZAR, 138, TRIANA - CENTRO</t>
         </is>
       </c>
       <c r="D453" s="2" t="inlineStr">
         <is>
-          <t>14B-041_PTZ_RUA FERNANDES BARRETOS AO LADO DA PREFEITURA</t>
+          <t>33-023_RF_TERMINAL RODOVIARIO DE VALENCA</t>
         </is>
       </c>
     </row>
@@ -10429,17 +10429,17 @@
       </c>
       <c r="B454" s="2" t="inlineStr">
         <is>
-          <t>CENTRO ESTADUAL EDUCAÇÃO PROF E SAÚDE DO L BAIANO-CEEP(ANTIGO COESVA)</t>
+          <t>CRECHE ESCOLA CASTELO DE AREIA</t>
         </is>
       </c>
       <c r="C454" s="2" t="inlineStr">
         <is>
-          <t>RUA FLORESTAL, 01 - BOLÍVIA</t>
+          <t>PRACA SAO JOSÉ 180 - GUAIBIM</t>
         </is>
       </c>
       <c r="D454" s="2" t="inlineStr">
         <is>
-          <t>33-039_PTZ_RUA DIRETA DA BOLIVIA_PRX DA IGREJA</t>
+          <t>33-010_PTZ_GUAIMBIM_PRAÇA SAO JOSE</t>
         </is>
       </c>
     </row>
@@ -10451,17 +10451,17 @@
       </c>
       <c r="B455" s="2" t="inlineStr">
         <is>
-          <t>COLÉGIO PERSPECTIVA</t>
+          <t>CRECHE ESCOLA CASTELO DE AREIA</t>
         </is>
       </c>
       <c r="C455" s="2" t="inlineStr">
         <is>
-          <t>PRAÇA CONSELHEIRO BALTAZAR, 138, TRIANA - CENTRO</t>
+          <t>PRACA SAO JOSÉ 180 - GUAIBIM</t>
         </is>
       </c>
       <c r="D455" s="2" t="inlineStr">
         <is>
-          <t>33-022_RF_TERMINAL RODOVIARIO DE VALENCA</t>
+          <t>33-011_PTZ_GUAIMBINZINHO_AV JOAO CLIMACO TEIXEIRA</t>
         </is>
       </c>
     </row>
@@ -10473,17 +10473,17 @@
       </c>
       <c r="B456" s="2" t="inlineStr">
         <is>
-          <t>COLÉGIO PERSPECTIVA</t>
+          <t>CRECHE ESCOLA CASTELO DE AREIA</t>
         </is>
       </c>
       <c r="C456" s="2" t="inlineStr">
         <is>
-          <t>PRAÇA CONSELHEIRO BALTAZAR, 138, TRIANA - CENTRO</t>
+          <t>PRACA SAO JOSÉ 180 - GUAIBIM</t>
         </is>
       </c>
       <c r="D456" s="2" t="inlineStr">
         <is>
-          <t>33-023_RF_TERMINAL RODOVIARIO DE VALENCA</t>
+          <t>33-033_RF_GUAIMBIM_PRX AO PONTO DE ONIBUS DA PRACA</t>
         </is>
       </c>
     </row>
@@ -10495,12 +10495,12 @@
       </c>
       <c r="B457" s="2" t="inlineStr">
         <is>
-          <t>CRECHE ESCOLA CASTELO DE AREIA</t>
+          <t>ESCOLA MUNICIPAL ALOÍSIO EVANGELISTA DA FONSECA</t>
         </is>
       </c>
       <c r="C457" s="2" t="inlineStr">
         <is>
-          <t>PRACA SAO JOSÉ 180 - GUAIBIM</t>
+          <t>RUA DO TAMARINEIRO, PRAÇA CENTRAL, S/N, ZONA RURAL</t>
         </is>
       </c>
       <c r="D457" s="2" t="inlineStr">
@@ -10517,17 +10517,17 @@
       </c>
       <c r="B458" s="2" t="inlineStr">
         <is>
-          <t>CRECHE ESCOLA CASTELO DE AREIA</t>
+          <t>ESCOLA MUNICIPAL ALOÍSIO EVANGELISTA DA FONSECA</t>
         </is>
       </c>
       <c r="C458" s="2" t="inlineStr">
         <is>
-          <t>PRACA SAO JOSÉ 180 - GUAIBIM</t>
+          <t>RUA DO TAMARINEIRO, PRAÇA CENTRAL, S/N, ZONA RURAL</t>
         </is>
       </c>
       <c r="D458" s="2" t="inlineStr">
         <is>
-          <t>33-011_PTZ_GUAIMBINZINHO_AV JOAO CLIMACO TEIXEIRA</t>
+          <t>33-033_RF_GUAIMBIM_PRX AO PONTO DE ONIBUS DA PRACA</t>
         </is>
       </c>
     </row>
@@ -10539,17 +10539,17 @@
       </c>
       <c r="B459" s="2" t="inlineStr">
         <is>
-          <t>CRECHE ESCOLA CASTELO DE AREIA</t>
+          <t>ESCOLA MUNICIPAL MANOEL SANTOS SILVA</t>
         </is>
       </c>
       <c r="C459" s="2" t="inlineStr">
         <is>
-          <t>PRACA SAO JOSÉ 180 - GUAIBIM</t>
+          <t>POVOADO BAIXÃO DO OROBÓ - POVOADO BAIXÃO DO OROBÓ</t>
         </is>
       </c>
       <c r="D459" s="2" t="inlineStr">
         <is>
-          <t>33-033_RF_GUAIMBIM_PRX AO PONTO DE ONIBUS DA PRACA</t>
+          <t>33-003_PTZ_RUA TEIXEIRA DE FREITAS_PROXIMO A LOJAS GUAIMBIM</t>
         </is>
       </c>
     </row>
@@ -10561,17 +10561,17 @@
       </c>
       <c r="B460" s="2" t="inlineStr">
         <is>
-          <t>ESCOLA MUNICIPAL ALOÍSIO EVANGELISTA DA FONSECA</t>
+          <t>ESCOLA MUNICIPAL MANOEL SANTOS SILVA</t>
         </is>
       </c>
       <c r="C460" s="2" t="inlineStr">
         <is>
-          <t>RUA DO TAMARINEIRO, PRAÇA CENTRAL, S/N, ZONA RURAL</t>
+          <t>POVOADO BAIXÃO DO OROBÓ - POVOADO BAIXÃO DO OROBÓ</t>
         </is>
       </c>
       <c r="D460" s="2" t="inlineStr">
         <is>
-          <t>33-010_PTZ_GUAIMBIM_PRAÇA SAO JOSE</t>
+          <t>33-004_PTZ_PRACA DA INDEPENDENCIA_PROXIMO AO BANCO DO BRASIL</t>
         </is>
       </c>
     </row>
@@ -10583,17 +10583,17 @@
       </c>
       <c r="B461" s="2" t="inlineStr">
         <is>
-          <t>ESCOLA MUNICIPAL ALOÍSIO EVANGELISTA DA FONSECA</t>
+          <t>ESCOLA MUNICIPAL MANOEL SANTOS SILVA</t>
         </is>
       </c>
       <c r="C461" s="2" t="inlineStr">
         <is>
-          <t>RUA DO TAMARINEIRO, PRAÇA CENTRAL, S/N, ZONA RURAL</t>
+          <t>POVOADO BAIXÃO DO OROBÓ - POVOADO BAIXÃO DO OROBÓ</t>
         </is>
       </c>
       <c r="D461" s="2" t="inlineStr">
         <is>
-          <t>33-033_RF_GUAIMBIM_PRX AO PONTO DE ONIBUS DA PRACA</t>
+          <t>33-026_RF_RUA DOM PEDRO II_PRX A OTICA PITUBA</t>
         </is>
       </c>
     </row>
@@ -10615,73 +10615,73 @@
       </c>
       <c r="D462" s="2" t="inlineStr">
         <is>
-          <t>33-003_PTZ_RUA TEIXEIRA DE FREITAS_PROXIMO A LOJAS GUAIMBIM</t>
+          <t>33-029_RF_CALCADAO_EM FRENTE_AO BANCO DO BRASIL</t>
         </is>
       </c>
     </row>
     <row r="463">
       <c r="A463" s="2" t="inlineStr">
         <is>
-          <t>VALENÇA</t>
+          <t>VERA CRUZ</t>
         </is>
       </c>
       <c r="B463" s="2" t="inlineStr">
         <is>
-          <t>ESCOLA MUNICIPAL MANOEL SANTOS SILVA</t>
+          <t>COMPLEXO CULTURAL ARISTÓTELES GOMES</t>
         </is>
       </c>
       <c r="C463" s="2" t="inlineStr">
         <is>
-          <t>POVOADO BAIXÃO DO OROBÓ - POVOADO BAIXÃO DO OROBÓ</t>
+          <t>RUA NOSSA SENHORA DAS CANDEIAS, S/N - ILHOTA</t>
         </is>
       </c>
       <c r="D463" s="2" t="inlineStr">
         <is>
-          <t>33-004_PTZ_PRACA DA INDEPENDENCIA_PROXIMO AO BANCO DO BRASIL</t>
+          <t>23B-049_LPR_RUA NOSSA SR DAS CANDEIAS STD ILHOTA VILAGE II</t>
         </is>
       </c>
     </row>
     <row r="464">
       <c r="A464" s="2" t="inlineStr">
         <is>
-          <t>VALENÇA</t>
+          <t>VERA CRUZ</t>
         </is>
       </c>
       <c r="B464" s="2" t="inlineStr">
         <is>
-          <t>ESCOLA MUNICIPAL MANOEL SANTOS SILVA</t>
+          <t>COMPLEXO CULTURAL ARISTÓTELES GOMES</t>
         </is>
       </c>
       <c r="C464" s="2" t="inlineStr">
         <is>
-          <t>POVOADO BAIXÃO DO OROBÓ - POVOADO BAIXÃO DO OROBÓ</t>
+          <t>RUA NOSSA SENHORA DAS CANDEIAS, S/N - ILHOTA</t>
         </is>
       </c>
       <c r="D464" s="2" t="inlineStr">
         <is>
-          <t>33-026_RF_RUA DOM PEDRO II_PRX A OTICA PITUBA</t>
+          <t>23B-073_PTZ_RUA NOSSA SR DAS CANDEIAS COMPLEXO CULTURAL ARISTOTELES GOMES</t>
         </is>
       </c>
     </row>
     <row r="465">
       <c r="A465" s="2" t="inlineStr">
         <is>
-          <t>VALENÇA</t>
+          <t>VERA CRUZ</t>
         </is>
       </c>
       <c r="B465" s="2" t="inlineStr">
         <is>
-          <t>ESCOLA MUNICIPAL MANOEL SANTOS SILVA</t>
+          <t>ESCOLA MUNICIPAL JORGE CALMON</t>
         </is>
       </c>
       <c r="C465" s="2" t="inlineStr">
         <is>
-          <t>POVOADO BAIXÃO DO OROBÓ - POVOADO BAIXÃO DO OROBÓ</t>
+          <t>RUA DIRETA DA COROA, S/N. - DISTRITO DE COROA</t>
         </is>
       </c>
       <c r="D465" s="2" t="inlineStr">
         <is>
-          <t>33-029_RF_CALCADAO_EM FRENTE_AO BANCO DO BRASIL</t>
+          <t>23B-050_LPR_BA 001 MAR GRANDE</t>
         </is>
       </c>
     </row>
@@ -10693,17 +10693,17 @@
       </c>
       <c r="B466" s="2" t="inlineStr">
         <is>
-          <t>COMPLEXO CULTURAL ARISTÓTELES GOMES</t>
+          <t>ESCOLA MUNICIPAL OLGA SEABRA</t>
         </is>
       </c>
       <c r="C466" s="2" t="inlineStr">
         <is>
-          <t>RUA NOSSA SENHORA DAS CANDEIAS, S/N - ILHOTA</t>
+          <t>RUA DO ARAÇÁ S/N - GAMBOA</t>
         </is>
       </c>
       <c r="D466" s="2" t="inlineStr">
         <is>
-          <t>23B-049_LPR_RUA NOSSA SR DAS CANDEIAS STD ILHOTA VILAGE II</t>
+          <t>23B-057_RF_TP_III_LADEIRA VINTE E OITO DE MAIO</t>
         </is>
       </c>
     </row>
@@ -10715,83 +10715,83 @@
       </c>
       <c r="B467" s="2" t="inlineStr">
         <is>
-          <t>COMPLEXO CULTURAL ARISTÓTELES GOMES</t>
+          <t>ESCOLA MUNICIPAL OLGA SEABRA</t>
         </is>
       </c>
       <c r="C467" s="2" t="inlineStr">
         <is>
-          <t>RUA NOSSA SENHORA DAS CANDEIAS, S/N - ILHOTA</t>
+          <t>RUA DO ARAÇÁ S/N - GAMBOA</t>
         </is>
       </c>
       <c r="D467" s="2" t="inlineStr">
         <is>
-          <t>23B-073_PTZ_RUA NOSSA SR DAS CANDEIAS COMPLEXO CULTURAL ARISTOTELES GOMES</t>
+          <t>23B-071_PTZ_LADEIRA VINTE E OITO DE MAIO AO LADO DO POSTO DE SAUDE DA GAMBOA</t>
         </is>
       </c>
     </row>
     <row r="468">
       <c r="A468" s="2" t="inlineStr">
         <is>
-          <t>VERA CRUZ</t>
+          <t>VITÓRIA DA CONQUISTA</t>
         </is>
       </c>
       <c r="B468" s="2" t="inlineStr">
         <is>
-          <t>ESCOLA MUNICIPAL JORGE CALMON</t>
+          <t>CAIC - CENTRO MUNICIPAL DE EDUCAÇÃO PROFESSOR PAULO FREIRE</t>
         </is>
       </c>
       <c r="C468" s="2" t="inlineStr">
         <is>
-          <t>RUA DIRETA DA COROA, S/N. - DISTRITO DE COROA</t>
+          <t>AVENIDA SÉRGIO VIEIRA DE MELLO, S/N - URBIS IV - ZABELÊ</t>
         </is>
       </c>
       <c r="D468" s="2" t="inlineStr">
         <is>
-          <t>23B-050_LPR_BA 001 MAR GRANDE</t>
+          <t>78-017_PTZ_AV_AMAZONAS_URBIS IV EM FRENTE A ESCOLA CAIC</t>
         </is>
       </c>
     </row>
     <row r="469">
       <c r="A469" s="2" t="inlineStr">
         <is>
-          <t>VERA CRUZ</t>
+          <t>VITÓRIA DA CONQUISTA</t>
         </is>
       </c>
       <c r="B469" s="2" t="inlineStr">
         <is>
-          <t>ESCOLA MUNICIPAL OLGA SEABRA</t>
+          <t>COLÉGIO DA POLÍCIA MILITAR ERALDO TINOCO</t>
         </is>
       </c>
       <c r="C469" s="2" t="inlineStr">
         <is>
-          <t>RUA DO ARAÇÁ S/N - GAMBOA</t>
+          <t>AVENIDA BRASÍLIA, 273  - PATAGÔNIA</t>
         </is>
       </c>
       <c r="D469" s="2" t="inlineStr">
         <is>
-          <t>23B-057_RF_TP_III_LADEIRA VINTE E OITO DE MAIO</t>
+          <t>78-023_RF_TP_IV_AV BRASILIA EM FRENTE AO COLEGIO CPM</t>
         </is>
       </c>
     </row>
     <row r="470">
       <c r="A470" s="2" t="inlineStr">
         <is>
-          <t>VERA CRUZ</t>
+          <t>VITÓRIA DA CONQUISTA</t>
         </is>
       </c>
       <c r="B470" s="2" t="inlineStr">
         <is>
-          <t>ESCOLA MUNICIPAL OLGA SEABRA</t>
+          <t>COLÉGIO ESTADUAL DOM CLIMÉRIO ALMEIDA DE ANDRADE</t>
         </is>
       </c>
       <c r="C470" s="2" t="inlineStr">
         <is>
-          <t>RUA DO ARAÇÁ S/N - GAMBOA</t>
+          <t>RUA F, Nº 987, URBIS IV, ESPÍRITO SANTO - ESPÍRITO SANTO</t>
         </is>
       </c>
       <c r="D470" s="2" t="inlineStr">
         <is>
-          <t>23B-071_PTZ_LADEIRA VINTE E OITO DE MAIO AO LADO DO POSTO DE SAUDE DA GAMBOA</t>
+          <t>77-025_PTZ_RUA A EM FRENTE A UNI DE SAUDE URBIS VI</t>
         </is>
       </c>
     </row>
@@ -10803,17 +10803,17 @@
       </c>
       <c r="B471" s="2" t="inlineStr">
         <is>
-          <t>CAIC - CENTRO MUNICIPAL DE EDUCAÇÃO PROFESSOR PAULO FREIRE</t>
+          <t>COLÉGIO ESTADUAL DOM CLIMÉRIO ALMEIDA DE ANDRADE</t>
         </is>
       </c>
       <c r="C471" s="2" t="inlineStr">
         <is>
-          <t>AVENIDA SÉRGIO VIEIRA DE MELLO, S/N - URBIS IV - ZABELÊ</t>
+          <t>RUA F, Nº 987, URBIS IV, ESPÍRITO SANTO - ESPÍRITO SANTO</t>
         </is>
       </c>
       <c r="D471" s="2" t="inlineStr">
         <is>
-          <t>78-017_PTZ_AV_AMAZONAS_URBIS IV EM FRENTE A ESCOLA CAIC</t>
+          <t>77-043_RF_TP_III_RUA A EM FRENTE A UNI DE SAUDE URBIS VI</t>
         </is>
       </c>
     </row>
@@ -10825,17 +10825,17 @@
       </c>
       <c r="B472" s="2" t="inlineStr">
         <is>
-          <t>COLÉGIO DA POLÍCIA MILITAR ERALDO TINOCO</t>
+          <t>COLÉGIO ESTADUAL PROFESSORA HELEUSA FIGUEIRA CÂMARA</t>
         </is>
       </c>
       <c r="C472" s="2" t="inlineStr">
         <is>
-          <t>AVENIDA BRASÍLIA, 273  - PATAGÔNIA</t>
+          <t>AVENIDA OLÍVIA FLORES, Nº 1180, CANDEIAS - CANDEIAS</t>
         </is>
       </c>
       <c r="D472" s="2" t="inlineStr">
         <is>
-          <t>78-023_RF_TP_IV_AV BRASILIA EM FRENTE AO COLEGIO CPM</t>
+          <t>77-022_PTZ_AV LUIS ED MAGALHAES EM FRENTE A ESCOLA PROF HELEUSA</t>
         </is>
       </c>
     </row>
@@ -10847,17 +10847,17 @@
       </c>
       <c r="B473" s="2" t="inlineStr">
         <is>
-          <t>COLÉGIO ESTADUAL DOM CLIMÉRIO ALMEIDA DE ANDRADE</t>
+          <t>ESCOLA MUNICIPAL FÉLIX PACHECO</t>
         </is>
       </c>
       <c r="C473" s="2" t="inlineStr">
         <is>
-          <t>RUA F, Nº 987, URBIS IV, ESPÍRITO SANTO - ESPÍRITO SANTO</t>
+          <t>POVOADO LAGOA DE JOSÉ LUIZ - DISTRITO DANTELÂNDIA</t>
         </is>
       </c>
       <c r="D473" s="2" t="inlineStr">
         <is>
-          <t>77-025_PTZ_RUA A EM FRENTE A UNI DE SAUDE URBIS VI</t>
+          <t>92-001_PTZ LAGOA JOSE LUIZ - COLEGIO MUNICIPAL FELIX PACHECO</t>
         </is>
       </c>
     </row>
@@ -10869,17 +10869,17 @@
       </c>
       <c r="B474" s="2" t="inlineStr">
         <is>
-          <t>COLÉGIO ESTADUAL DOM CLIMÉRIO ALMEIDA DE ANDRADE</t>
+          <t>ESCOLA MUNICIPAL JOSÉ MOZART TANAJURA</t>
         </is>
       </c>
       <c r="C474" s="2" t="inlineStr">
         <is>
-          <t>RUA F, Nº 987, URBIS IV, ESPÍRITO SANTO - ESPÍRITO SANTO</t>
+          <t>RUA SÉRGIO BUARQUE DE HOLANDA, N 2000, VILA AMÉRICA - BOA VISTA</t>
         </is>
       </c>
       <c r="D474" s="2" t="inlineStr">
         <is>
-          <t>77-043_RF_TP_III_RUA A EM FRENTE A UNI DE SAUDE URBIS VI</t>
+          <t>77-016_PTZ_RUA JUSCELINO KUBITSCHEK EM FRENTE A UNIAO CASA DE CARNES VILA AMERICA</t>
         </is>
       </c>
     </row>
@@ -10891,17 +10891,17 @@
       </c>
       <c r="B475" s="2" t="inlineStr">
         <is>
-          <t>COLÉGIO ESTADUAL PROFESSORA HELEUSA FIGUEIRA CÂMARA</t>
+          <t>ESCOLA MUNICIPAL LIONS CLUBE</t>
         </is>
       </c>
       <c r="C475" s="2" t="inlineStr">
         <is>
-          <t>AVENIDA OLÍVIA FLORES, Nº 1180, CANDEIAS - CANDEIAS</t>
+          <t>AVENIDA SERRINHA, 2284 - BRASIL</t>
         </is>
       </c>
       <c r="D475" s="2" t="inlineStr">
         <is>
-          <t>77-022_PTZ_AV LUIS ED MAGALHAES EM FRENTE A ESCOLA PROF HELEUSA</t>
+          <t>78-009_PTZ_AV ALAGOAS EM FRENTE AO SUP MERCADO ECONOMIA</t>
         </is>
       </c>
     </row>
@@ -10913,17 +10913,17 @@
       </c>
       <c r="B476" s="2" t="inlineStr">
         <is>
-          <t>ESCOLA MUNICIPAL FÉLIX PACHECO</t>
+          <t>ESCOLA MUNICIPAL LYCIA PEDRAL</t>
         </is>
       </c>
       <c r="C476" s="2" t="inlineStr">
         <is>
-          <t>POVOADO LAGOA DE JOSÉ LUIZ - DISTRITO DANTELÂNDIA</t>
+          <t>AVENIDA ROSA CRUZ, S/N, ALTO MARON - ALTO MARON</t>
         </is>
       </c>
       <c r="D476" s="2" t="inlineStr">
         <is>
-          <t>92-001_PTZ LAGOA JOSE LUIZ - COLEGIO MUNICIPAL FELIX PACHECO</t>
+          <t>77-027_PTZ_RUA BELA VISTA EM FRENTE ESCOLA LYCIA PEDRAL-SANTA CECILIA</t>
         </is>
       </c>
     </row>
@@ -10935,17 +10935,17 @@
       </c>
       <c r="B477" s="2" t="inlineStr">
         <is>
-          <t>ESCOLA MUNICIPAL JOSÉ MOZART TANAJURA</t>
+          <t>ESCOLA MUNICIPAL PAULO SETÚBAL</t>
         </is>
       </c>
       <c r="C477" s="2" t="inlineStr">
         <is>
-          <t>RUA SÉRGIO BUARQUE DE HOLANDA, N 2000, VILA AMÉRICA - BOA VISTA</t>
+          <t>DISTRITO INHOBIM - DISTRITO INHOBIM</t>
         </is>
       </c>
       <c r="D477" s="2" t="inlineStr">
         <is>
-          <t>77-016_PTZ_RUA JUSCELINO KUBITSCHEK EM FRENTE A UNIAO CASA DE CARNES VILA AMERICA</t>
+          <t>92-015_RF_TP_III_RUA DURVAL SANTOS_INHOBIM_AO LADO DA FARMACIA</t>
         </is>
       </c>
     </row>
@@ -10957,17 +10957,17 @@
       </c>
       <c r="B478" s="2" t="inlineStr">
         <is>
-          <t>ESCOLA MUNICIPAL LIONS CLUBE</t>
+          <t>ESCOLA MUNICIPAL PROFESSORA MARLENE FLORES</t>
         </is>
       </c>
       <c r="C478" s="2" t="inlineStr">
         <is>
-          <t>AVENIDA SERRINHA, 2284 - BRASIL</t>
+          <t>RUA MARGARIDA OLIVEIRA CUNHA, S/N, LAGOA DAS FLORES - LAGOA DAS FLORES</t>
         </is>
       </c>
       <c r="D478" s="2" t="inlineStr">
         <is>
-          <t>78-009_PTZ_AV ALAGOAS EM FRENTE AO SUP MERCADO ECONOMIA</t>
+          <t>92-016_PTZ_FRENTE A ESCOLA PROF MARLENE FLORES_LAGOA DAS FLORES</t>
         </is>
       </c>
     </row>
@@ -10979,17 +10979,17 @@
       </c>
       <c r="B479" s="2" t="inlineStr">
         <is>
-          <t>ESCOLA MUNICIPAL LYCIA PEDRAL</t>
+          <t>ESCOLA MUNICIPAL VICENTE CASSIMIRO</t>
         </is>
       </c>
       <c r="C479" s="2" t="inlineStr">
         <is>
-          <t>AVENIDA ROSA CRUZ, S/N, ALTO MARON - ALTO MARON</t>
+          <t>ESTRADA BEM QUERER, KM 4, UNIVERSIDADE- UNIVERSIDADE</t>
         </is>
       </c>
       <c r="D479" s="2" t="inlineStr">
         <is>
-          <t>77-027_PTZ_RUA BELA VISTA EM FRENTE ESCOLA LYCIA PEDRAL-SANTA CECILIA</t>
+          <t>77-065_RF_TP_IV AV EDMUNDO SILVEIRA FLORES-ENTRADA DA UESB</t>
         </is>
       </c>
     </row>
@@ -11001,17 +11001,17 @@
       </c>
       <c r="B480" s="2" t="inlineStr">
         <is>
-          <t>ESCOLA MUNICIPAL PAULO SETÚBAL</t>
+          <t>FACULDADE ANHANGUERA - VITÓRIA DA CONQUISTA</t>
         </is>
       </c>
       <c r="C480" s="2" t="inlineStr">
         <is>
-          <t>DISTRITO INHOBIM - DISTRITO INHOBIM</t>
+          <t>AVENIDA JURACY MAGALHÃES, 3000 - BOA VISTA</t>
         </is>
       </c>
       <c r="D480" s="2" t="inlineStr">
         <is>
-          <t>92-015_RF_TP_III_RUA DURVAL SANTOS_INHOBIM_AO LADO DA FARMACIA</t>
+          <t>77-047_RF_TP_IV_AV JURACY MAGALHAES EM FRENTE AO SHOP CONQUISTA SUL</t>
         </is>
       </c>
     </row>
@@ -11023,17 +11023,17 @@
       </c>
       <c r="B481" s="2" t="inlineStr">
         <is>
-          <t>ESCOLA MUNICIPAL PROFESSORA MARLENE FLORES</t>
+          <t>FACULDADE ANHANGUERA - VITÓRIA DA CONQUISTA</t>
         </is>
       </c>
       <c r="C481" s="2" t="inlineStr">
         <is>
-          <t>RUA MARGARIDA OLIVEIRA CUNHA, S/N, LAGOA DAS FLORES - LAGOA DAS FLORES</t>
+          <t>AVENIDA JURACY MAGALHÃES, 3000 - BOA VISTA</t>
         </is>
       </c>
       <c r="D481" s="2" t="inlineStr">
         <is>
-          <t>92-016_PTZ_FRENTE A ESCOLA PROF MARLENE FLORES_LAGOA DAS FLORES</t>
+          <t>77-055_RF_TP_IV_AV JURACY MAGALHAES AO LADO DA FACUL PITAGORAS</t>
         </is>
       </c>
     </row>
@@ -11045,17 +11045,17 @@
       </c>
       <c r="B482" s="2" t="inlineStr">
         <is>
-          <t>ESCOLA MUNICIPAL VICENTE CASSIMIRO</t>
+          <t>PREFEITURA MUNICIPAL DE VITÓRIA DA CONQUISTA</t>
         </is>
       </c>
       <c r="C482" s="2" t="inlineStr">
         <is>
-          <t>ESTRADA BEM QUERER, KM 4, UNIVERSIDADE- UNIVERSIDADE</t>
+          <t>PRAÇA JOAQUIM CORREIA, Nº 55, CENTRO - CENTRO</t>
         </is>
       </c>
       <c r="D482" s="2" t="inlineStr">
         <is>
-          <t>77-065_RF_TP_IV AV EDMUNDO SILVEIRA FLORES-ENTRADA DA UESB</t>
+          <t>77-117_PTZ_PRACA JOAQUIM CORREIA_PREFEITURA</t>
         </is>
       </c>
     </row>
@@ -11067,17 +11067,17 @@
       </c>
       <c r="B483" s="2" t="inlineStr">
         <is>
-          <t>FACULDADE ANHANGUERA - VITÓRIA DA CONQUISTA</t>
+          <t>PREFEITURA MUNICIPAL DE VITÓRIA DA CONQUISTA</t>
         </is>
       </c>
       <c r="C483" s="2" t="inlineStr">
         <is>
-          <t>AVENIDA JURACY MAGALHÃES, 3000 - BOA VISTA</t>
+          <t>PRAÇA JOAQUIM CORREIA, Nº 55, CENTRO - CENTRO</t>
         </is>
       </c>
       <c r="D483" s="2" t="inlineStr">
         <is>
-          <t>77-047_RF_TP_IV_AV JURACY MAGALHAES EM FRENTE AO SHOP CONQUISTA SUL</t>
+          <t>77-136_RF_TP_IV_PRACA JOAQUIM CORREIA</t>
         </is>
       </c>
     </row>
@@ -11089,17 +11089,17 @@
       </c>
       <c r="B484" s="2" t="inlineStr">
         <is>
-          <t>FACULDADE ANHANGUERA - VITÓRIA DA CONQUISTA</t>
+          <t>PREFEITURA MUNICIPAL DE VITÓRIA DA CONQUISTA</t>
         </is>
       </c>
       <c r="C484" s="2" t="inlineStr">
         <is>
-          <t>AVENIDA JURACY MAGALHÃES, 3000 - BOA VISTA</t>
+          <t>PRAÇA JOAQUIM CORREIA, Nº 55, CENTRO - CENTRO</t>
         </is>
       </c>
       <c r="D484" s="2" t="inlineStr">
         <is>
-          <t>77-055_RF_TP_IV_AV JURACY MAGALHAES AO LADO DA FACUL PITAGORAS</t>
+          <t>77-148_PTZ_R DOS ANDRADES CENTRO</t>
         </is>
       </c>
     </row>
@@ -11111,17 +11111,17 @@
       </c>
       <c r="B485" s="2" t="inlineStr">
         <is>
-          <t>PREFEITURA MUNICIPAL DE VITÓRIA DA CONQUISTA</t>
+          <t>UNEX - CENTRO UNIVERSITÁRIO DE EXCELÊNCIA (ANTIGA UNIFTC)</t>
         </is>
       </c>
       <c r="C485" s="2" t="inlineStr">
         <is>
-          <t>PRAÇA JOAQUIM CORREIA, Nº 55, CENTRO - CENTRO</t>
+          <t>RUA UBALDINO FIGUEIRA, Nº 200, RECREIO - RECREIO</t>
         </is>
       </c>
       <c r="D485" s="2" t="inlineStr">
         <is>
-          <t>77-117_PTZ_PRACA JOAQUIM CORREIA_PREFEITURA</t>
+          <t>77-012_PTZ_AV LEONIDIO OLIVEIRA EM FRENTE A UNIFTC</t>
         </is>
       </c>
     </row>
@@ -11133,125 +11133,59 @@
       </c>
       <c r="B486" s="2" t="inlineStr">
         <is>
-          <t>PREFEITURA MUNICIPAL DE VITÓRIA DA CONQUISTA</t>
+          <t>UNEX - CENTRO UNIVERSITÁRIO DE EXCELÊNCIA (ANTIGA UNIFTC)</t>
         </is>
       </c>
       <c r="C486" s="2" t="inlineStr">
         <is>
-          <t>PRAÇA JOAQUIM CORREIA, Nº 55, CENTRO - CENTRO</t>
+          <t>RUA UBALDINO FIGUEIRA, Nº 200, RECREIO - RECREIO</t>
         </is>
       </c>
       <c r="D486" s="2" t="inlineStr">
         <is>
-          <t>77-136_RF_TP_IV_PRACA JOAQUIM CORREIA</t>
+          <t>77-064_RF_TP_IV_AV LEONIDIO OLIVEIRA PROXIMO AO UNIFTC</t>
         </is>
       </c>
     </row>
     <row r="487">
       <c r="A487" s="2" t="inlineStr">
         <is>
-          <t>VITÓRIA DA CONQUISTA</t>
+          <t>ÉRICO CARDOSO</t>
         </is>
       </c>
       <c r="B487" s="2" t="inlineStr">
         <is>
-          <t>PREFEITURA MUNICIPAL DE VITÓRIA DA CONQUISTA</t>
+          <t>COLÉGIO ANTÔNIO CARLOS MAGALHÃES</t>
         </is>
       </c>
       <c r="C487" s="2" t="inlineStr">
         <is>
-          <t>PRAÇA JOAQUIM CORREIA, Nº 55, CENTRO - CENTRO</t>
+          <t>AVENIDA ANTÔNIO CARLOS MAGALHÃES - CENTRO</t>
         </is>
       </c>
       <c r="D487" s="2" t="inlineStr">
         <is>
-          <t>77-148_PTZ_R DOS ANDRADES CENTRO</t>
+          <t>46-002_PTZ_AV ACM EM FRENTE A APAE</t>
         </is>
       </c>
     </row>
     <row r="488">
       <c r="A488" s="2" t="inlineStr">
         <is>
-          <t>VITÓRIA DA CONQUISTA</t>
+          <t>ÉRICO CARDOSO</t>
         </is>
       </c>
       <c r="B488" s="2" t="inlineStr">
         <is>
-          <t>UNEX - CENTRO UNIVERSITÁRIO DE EXCELÊNCIA (ANTIGA UNIFTC)</t>
+          <t>COLÉGIO ANTÔNIO CARLOS MAGALHÃES</t>
         </is>
       </c>
       <c r="C488" s="2" t="inlineStr">
         <is>
-          <t>RUA UBALDINO FIGUEIRA, Nº 200, RECREIO - RECREIO</t>
+          <t>AVENIDA ANTÔNIO CARLOS MAGALHÃES - CENTRO</t>
         </is>
       </c>
       <c r="D488" s="2" t="inlineStr">
-        <is>
-          <t>77-012_PTZ_AV LEONIDIO OLIVEIRA EM FRENTE A UNIFTC</t>
-        </is>
-      </c>
-    </row>
-    <row r="489">
-      <c r="A489" s="2" t="inlineStr">
-        <is>
-          <t>VITÓRIA DA CONQUISTA</t>
-        </is>
-      </c>
-      <c r="B489" s="2" t="inlineStr">
-        <is>
-          <t>UNEX - CENTRO UNIVERSITÁRIO DE EXCELÊNCIA (ANTIGA UNIFTC)</t>
-        </is>
-      </c>
-      <c r="C489" s="2" t="inlineStr">
-        <is>
-          <t>RUA UBALDINO FIGUEIRA, Nº 200, RECREIO - RECREIO</t>
-        </is>
-      </c>
-      <c r="D489" s="2" t="inlineStr">
-        <is>
-          <t>77-064_RF_TP_IV_AV LEONIDIO OLIVEIRA PROXIMO AO UNIFTC</t>
-        </is>
-      </c>
-    </row>
-    <row r="490">
-      <c r="A490" s="2" t="inlineStr">
-        <is>
-          <t>ÉRICO CARDOSO</t>
-        </is>
-      </c>
-      <c r="B490" s="2" t="inlineStr">
-        <is>
-          <t>COLÉGIO ANTÔNIO CARLOS MAGALHÃES</t>
-        </is>
-      </c>
-      <c r="C490" s="2" t="inlineStr">
-        <is>
-          <t>AVENIDA ANTÔNIO CARLOS MAGALHÃES - CENTRO</t>
-        </is>
-      </c>
-      <c r="D490" s="2" t="inlineStr">
-        <is>
-          <t>46-002_PTZ_AV ACM EM FRENTE A APAE</t>
-        </is>
-      </c>
-    </row>
-    <row r="491">
-      <c r="A491" s="2" t="inlineStr">
-        <is>
-          <t>ÉRICO CARDOSO</t>
-        </is>
-      </c>
-      <c r="B491" s="2" t="inlineStr">
-        <is>
-          <t>COLÉGIO ANTÔNIO CARLOS MAGALHÃES</t>
-        </is>
-      </c>
-      <c r="C491" s="2" t="inlineStr">
-        <is>
-          <t>AVENIDA ANTÔNIO CARLOS MAGALHÃES - CENTRO</t>
-        </is>
-      </c>
-      <c r="D491" s="2" t="inlineStr">
         <is>
           <t>46-011_RF_TP_IV_AV ACM EM FRENTE A ESCOLA ESTADUAL DE ERICO CARDO</t>
         </is>

</xml_diff>